<commit_message>
Document saved Rev-E1 hull leakage repairs and build holds
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Energized Water Scanner" sheetId="1" r:id="R5eed4888be374821"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Energized Water Scanner" sheetId="1" r:id="R0d13f7dd973b480e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -532,7 +532,7 @@
         <x:v>RC boat</x:v>
       </x:c>
       <x:c r="H5" s="15" t="str">
-        <x:v>Rev E | 28 Sep 2026</x:v>
+        <x:v>Rev E1, 29 Sep 2026</x:v>
       </x:c>
       <x:c r="I5" s="15"/>
       <x:c r="J5" s="15"/>
@@ -611,10 +611,10 @@
       <x:c r="I7" s="15"/>
       <x:c r="J7" s="15"/>
       <x:c r="K7" s="15" t="str">
-        <x:v>Fit verification required</x:v>
+        <x:v>HOLD: internal shaft sealing</x:v>
       </x:c>
       <x:c r="L7" s="15" t="str">
-        <x:v>Existing sheet price estimate retained; not a verified current quotation.</x:v>
+        <x:v>Qualify shaft-to-tube sealing/lubrication separately from hull bond. Price estimate unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="66" customHeight="1">
@@ -1626,7 +1626,7 @@
         <x:v>Fit verification required</x:v>
       </x:c>
       <x:c r="L41" s="14" t="str">
-        <x:v>Starting length; verify flange/gasket engagement and sealing preload.</x:v>
+        <x:v>Rev E1: 3 mm flange + 0.75 mm gasket; 5 mm pilot. M3x8 gives 4.25 mm engagement, 0.75 mm tip gap. Verify.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="66" customHeight="1">
@@ -2018,7 +2018,7 @@
         <x:v>Fit verification required</x:v>
       </x:c>
       <x:c r="L55" s="15" t="str">
-        <x:v>Select final length and seal penetration if applicable.</x:v>
+        <x:v>Rev E1: bores stop at X=193 mm, with 3 mm caps. Select length for tip X&gt;=193.75 mm; verify engagement.</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="66" customHeight="1">
@@ -2260,7 +2260,7 @@
         <x:f>IF(C64="","",B64*D64)</x:f>
       </x:c>
       <x:c r="F64" s="13" t="str">
-        <x:v>prints/Print_STLs.zip</x:v>
+        <x:v>docs/RevE1_Changes.md</x:v>
       </x:c>
       <x:c r="G64" s="13" t="str">
         <x:v>Both</x:v>
@@ -2269,10 +2269,10 @@
       <x:c r="I64" s="13"/>
       <x:c r="J64" s="13"/>
       <x:c r="K64" s="13" t="str">
-        <x:v>Print and qualify</x:v>
+        <x:v>HOLD: new hull export</x:v>
       </x:c>
       <x:c r="L64" s="13" t="str">
-        <x:v>Current Rev-E STL; unfilled insulating PETG fit prototype. Do not scale.</x:v>
+        <x:v>Rev E1 repairs wall and blind screw bores; trims obsolete foot. Existing Rev E hull STL is stale.</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="66" customHeight="1">

</xml_diff>